<commit_message>
changed excel -add class Cell | value -add type dateTime -auto write type cell
</commit_message>
<xml_diff>
--- a/тест/test.xlsx
+++ b/тест/test.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сотрудники" sheetId="1" r:id="R22db2962dc5f4d6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сотрудники" sheetId="1" r:id="R1a99809dfaa94f2f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -34,6 +34,10 @@
     <x:t>02.10.2010</x:t>
   </x:si>
 </x:sst>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
bug fixed change data type excel
</commit_message>
<xml_diff>
--- a/тест/test.xlsx
+++ b/тест/test.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сотрудники" sheetId="1" r:id="R1a99809dfaa94f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сотрудники" sheetId="1" r:id="Rd5346ed0452b44ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -27,17 +27,45 @@
   <x:si>
     <x:t>Фронтенщик</x:t>
   </x:si>
-  <x:si>
-    <x:t>01.01.1999</x:t>
-  </x:si>
-  <x:si>
-    <x:t>02.10.2010</x:t>
-  </x:si>
 </x:sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts>
+    <x:numFmt numFmtId="14" formatCode="dd.mm.yyyy"/>
+  </x:numFmts>
+  <x:fonts>
+    <x:font>
+      <x:sz val="11"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:charset val="204"/>
+      <x:scheme val="minor"/>
+    </x:font>
+  </x:fonts>
+  <x:fills>
+    <x:fill>
+      <x:patternFill patternType="none"/>
+    </x:fill>
+  </x:fills>
+  <x:borders>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="0"/>
+    <x:xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  </x:cellXfs>
+</x:styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -71,11 +99,11 @@
       <x:c r="B2" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="C2" t="s">
-        <x:v>6</x:v>
+      <x:c r="C2" s="1">
+        <x:v>36506</x:v>
       </x:c>
-      <x:c r="D2" t="s">
-        <x:v>7</x:v>
+      <x:c r="D2" s="1">
+        <x:v>46083,42542824074</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>